<commit_message>
Add customer toggle - switch between Airtel Africa/OBF and MTN
</commit_message>
<xml_diff>
--- a/Issue Tracker AA_OBF.xlsx
+++ b/Issue Tracker AA_OBF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\eknriis\DELETE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{281A3085-1C26-4655-BC22-C69BA886193F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80A216DB-DBBE-405C-8D8F-C4C1D2DDF3DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{94F30213-8432-4ADA-9844-C97DB16F3E88}"/>
   </bookViews>
@@ -305,9 +305,6 @@
     <t xml:space="preserve">Airtel East </t>
   </si>
   <si>
-    <t>Issue suspected at customer network end. RCA awaited</t>
-  </si>
-  <si>
     <t>REQ000002086776</t>
   </si>
   <si>
@@ -622,6 +619,9 @@
   <si>
     <t>06/09/2026, 01:30 AM</t>
   </si>
+  <si>
+    <t>Issue suspected at customer network end</t>
+  </si>
 </sst>
 </file>
 
@@ -630,7 +630,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="[hh]:mm"/>
-    <numFmt numFmtId="174" formatCode="dd\/mm\/yyyy\ hh:mm\ AM/PM"/>
+    <numFmt numFmtId="166" formatCode="dd\/mm\/yyyy\ hh:mm\ AM/PM"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -664,18 +664,19 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -766,7 +767,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -792,8 +793,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="7" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
@@ -860,7 +860,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="174" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="22" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -888,19 +888,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="14" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1272,773 +1260,773 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="J1" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="K1" s="17" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="22">
+      <c r="A2" s="21">
         <v>46145</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="23" t="s">
+      <c r="D2" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="23" t="s">
+      <c r="G2" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="23" t="s">
+      <c r="H2" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="21">
+        <v>46146</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="I2" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" s="15" t="s">
+      <c r="I3" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="15" t="s">
+      <c r="K3" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="21">
+        <v>46147</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="H4" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="21">
+        <v>46162</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="K5" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="21">
+        <v>46162</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="J6" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="K6" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="21">
+        <v>46185</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="21">
+        <v>46177</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="G8" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="H8" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="I8" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="21">
+        <v>46178</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="H9" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="J9" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="21">
+        <v>46179</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="H10" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="I10" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="J10" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="K10" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="21">
+        <v>46184</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="H11" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="I11" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="J11" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="K11" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="21">
+        <v>46190</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="G12" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="H12" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="J12" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="K12" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="21">
+        <v>46198</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="G13" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="H13" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="I13" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="J13" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="K13" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="21">
+        <v>46200</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="H14" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="J14" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="K14" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="21">
+        <v>46201</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="G15" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="H15" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="J15" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="K15" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="21">
+        <v>46203</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="H16" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="J16" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="21">
+        <v>46204</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="G17" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="H17" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="21">
+        <v>46204</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="H18" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="I18" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="J18" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="K18" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="21">
+        <v>46211</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>113</v>
+      </c>
+      <c r="G19" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="H19" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="I19" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="J19" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="K19" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="21">
+        <v>46211</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="H20" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="I20" s="14" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="22">
-        <v>46146</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="I3" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22">
-        <v>46147</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="23" t="s">
+      <c r="J20" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="K20" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="21">
+        <v>46253</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="G21" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="H21" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="J21" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="K21" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" s="21">
+        <v>46255</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="H4" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="I4" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="J4" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="K4" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="22">
-        <v>46162</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="K5" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="22">
-        <v>46162</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="H6" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="I6" s="16" t="s">
-        <v>157</v>
-      </c>
-      <c r="J6" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="K6" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="22">
-        <v>46185</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="H7" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="I7" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="J7" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="K7" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="22">
-        <v>46177</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="23" t="s">
-        <v>98</v>
-      </c>
-      <c r="G8" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="H8" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="I8" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="J8" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="K8" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="22">
-        <v>46178</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="G9" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="H9" s="23" t="s">
-        <v>135</v>
-      </c>
-      <c r="I9" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="J9" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="K9" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="22">
-        <v>46179</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="H10" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="I10" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="J10" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="K10" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="22">
-        <v>46184</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="G11" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="H11" s="23" t="s">
-        <v>137</v>
-      </c>
-      <c r="I11" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="J11" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="K11" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="22">
-        <v>46190</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="G12" s="23" t="s">
-        <v>105</v>
-      </c>
-      <c r="H12" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="I12" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="J12" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="K12" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="22">
-        <v>46198</v>
-      </c>
-      <c r="B13" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="23" t="s">
-        <v>106</v>
-      </c>
-      <c r="G13" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="H13" s="23" t="s">
-        <v>139</v>
-      </c>
-      <c r="I13" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="J13" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="K13" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="22">
-        <v>46200</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="G14" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="H14" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="I14" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="J14" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="K14" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="22">
-        <v>46201</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="G15" s="24" t="s">
-        <v>109</v>
-      </c>
-      <c r="H15" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="I15" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="J15" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="K15" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="22">
-        <v>46203</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D16" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="23" t="s">
-        <v>126</v>
-      </c>
-      <c r="G16" s="24" t="s">
-        <v>127</v>
-      </c>
-      <c r="H16" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="I16" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="J16" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="K16" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="22">
-        <v>46204</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="G17" s="25" t="s">
-        <v>111</v>
-      </c>
-      <c r="H17" s="23" t="s">
-        <v>143</v>
-      </c>
-      <c r="I17" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="J17" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="K17" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A18" s="22">
-        <v>46204</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F18" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="G18" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="H18" s="23" t="s">
-        <v>144</v>
-      </c>
-      <c r="I18" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="J18" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="K18" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" s="22">
-        <v>46211</v>
-      </c>
-      <c r="B19" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="G19" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="H19" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="I19" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="J19" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="K19" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" s="22">
-        <v>46211</v>
-      </c>
-      <c r="B20" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E20" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F20" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="G20" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="H20" s="23" t="s">
-        <v>135</v>
-      </c>
-      <c r="I20" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="J20" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="K20" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A21" s="22">
-        <v>46253</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="C21" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F21" s="23" t="s">
+      <c r="D22" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="G21" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="H21" s="26" t="s">
+      <c r="G22" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="H22" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="I21" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="J21" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="K21" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" s="22">
-        <v>46255</v>
-      </c>
-      <c r="B22" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E22" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="G22" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="H22" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="I22" s="15" t="s">
+      <c r="I22" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="J22" s="15" t="s">
+      <c r="J22" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="K22" s="15" t="s">
-        <v>87</v>
+      <c r="K22" s="14" t="s">
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -2064,139 +2052,137 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="J1" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="22">
+      <c r="A2" s="21">
         <v>46157</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="28" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="28" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="28" t="s">
+      <c r="C2" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="F2" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="H2" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="J2" s="22" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="28">
+        <v>46185</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="30">
+        <v>46362.495138888888</v>
+      </c>
+      <c r="F3" s="30">
+        <v>46362.564583333333</v>
+      </c>
+      <c r="G3" s="27" t="s">
+        <v>150</v>
+      </c>
+      <c r="H3" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="I3" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="J3" s="22" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="28">
+        <v>46186</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="31" t="s">
+        <v>151</v>
+      </c>
+      <c r="F4" s="31" t="s">
         <v>153</v>
       </c>
-      <c r="F2" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="28" t="s">
+      <c r="G4" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="H2" s="27" t="s">
+      <c r="H4" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="I2" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="J2" s="23" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="29">
-        <v>46185</v>
-      </c>
-      <c r="B3" s="30" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="30" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="31">
-        <v>46362.495138888888</v>
-      </c>
-      <c r="F3" s="31">
-        <v>46362.564583333333</v>
-      </c>
-      <c r="G3" s="28" t="s">
-        <v>151</v>
-      </c>
-      <c r="H3" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="I3" s="23" t="s">
+      <c r="I4" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="J3" s="23" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="29">
-        <v>46186</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="32" t="s">
-        <v>152</v>
-      </c>
-      <c r="F4" s="32" t="s">
-        <v>154</v>
-      </c>
-      <c r="G4" s="28" t="s">
-        <v>149</v>
-      </c>
-      <c r="H4" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="I4" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="J4" s="23" t="s">
+      <c r="J4" s="22" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2220,66 +2206,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="E1" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="F1" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="36" t="s">
+      <c r="G1" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="37" t="s">
+      <c r="H1" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="35" t="s">
+      <c r="I1" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="J1" s="38" t="s">
+      <c r="J1" s="37" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="39">
+      <c r="A2" s="32">
         <v>46181</v>
       </c>
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="40" t="s">
+      <c r="C2" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="40" t="s">
+      <c r="D2" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="41" t="s">
+      <c r="E2" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="G2" s="23" t="s">
         <v>160</v>
       </c>
-      <c r="G2" s="41" t="s">
-        <v>161</v>
-      </c>
-      <c r="H2" s="43" t="s">
-        <v>150</v>
-      </c>
-      <c r="I2" s="42" t="s">
-        <v>97</v>
-      </c>
-      <c r="J2" s="40"/>
+      <c r="H2" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="J2" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2304,34 +2290,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="J1" s="13" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2368,130 +2354,130 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="I1" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="J1" s="20" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="33">
+      <c r="A2" s="32">
         <v>46176</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="G2" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="H2" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="I2" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="J2" s="26" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="32">
+        <v>46179</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="C2" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="23" t="s">
+      <c r="G3" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="I3" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="J3" s="26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="21">
+        <v>46200</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="G2" s="23" t="s">
-        <v>168</v>
-      </c>
-      <c r="H2" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="I2" s="27" t="s">
+      <c r="G4" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="H4" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="I4" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="J2" s="27" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="33">
-        <v>46179</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D3" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="23" t="s">
-        <v>163</v>
-      </c>
-      <c r="G3" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="H3" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="I3" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="J3" s="27" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="22">
-        <v>46200</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="C4" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="D4" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>165</v>
-      </c>
-      <c r="G4" s="23" t="s">
-        <v>166</v>
-      </c>
-      <c r="H4" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="I4" s="27" t="s">
-        <v>66</v>
-      </c>
-      <c r="J4" s="27" t="s">
+      <c r="J4" s="26" t="s">
         <v>72</v>
       </c>
     </row>
@@ -2518,162 +2504,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="J1" s="13" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="22">
+      <c r="A2" s="21">
         <v>46197</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="23" t="s">
+      <c r="D2" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>171</v>
+      </c>
+      <c r="G2" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="H2" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="I2" s="40" t="s">
+        <v>75</v>
+      </c>
+      <c r="J2" s="41" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="21">
+        <v>46203</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="G3" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="I3" s="40" t="s">
+        <v>93</v>
+      </c>
+      <c r="J3" s="41" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="21">
+        <v>46205</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="G4" s="22" t="s">
         <v>172</v>
       </c>
-      <c r="G2" s="23" t="s">
-        <v>175</v>
-      </c>
-      <c r="H2" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="I2" s="45" t="s">
+      <c r="H4" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="I4" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="J4" s="41" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="21">
+        <v>46241</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="33" t="s">
+        <v>169</v>
+      </c>
+      <c r="G5" s="33" t="s">
+        <v>173</v>
+      </c>
+      <c r="H5" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="I5" s="42" t="s">
         <v>75</v>
       </c>
-      <c r="J2" s="46" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="22">
-        <v>46203</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="G3" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="H3" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="I3" s="45" t="s">
-        <v>94</v>
-      </c>
-      <c r="J3" s="46" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="22">
-        <v>46205</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>169</v>
-      </c>
-      <c r="G4" s="23" t="s">
-        <v>173</v>
-      </c>
-      <c r="H4" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="I4" s="45" t="s">
-        <v>91</v>
-      </c>
-      <c r="J4" s="46" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="22">
-        <v>46241</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="34" t="s">
-        <v>170</v>
-      </c>
-      <c r="G5" s="34" t="s">
-        <v>174</v>
-      </c>
-      <c r="H5" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="I5" s="47" t="s">
-        <v>75</v>
-      </c>
-      <c r="J5" s="48" t="s">
+      <c r="J5" s="43" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2704,66 +2690,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="J1" s="17" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="44">
+      <c r="A2" s="39">
         <v>46182</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="28" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="28" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="28" t="s">
+      <c r="D2" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="27" t="s">
+        <v>176</v>
+      </c>
+      <c r="G2" s="27" t="s">
         <v>177</v>
       </c>
-      <c r="G2" s="28" t="s">
-        <v>178</v>
-      </c>
-      <c r="H2" s="27" t="s">
+      <c r="H2" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="I2" s="49" t="s">
+      <c r="I2" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="J2" s="50" t="s">
+      <c r="J2" s="45" t="s">
         <v>84</v>
       </c>
     </row>
@@ -2773,6 +2759,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ED8B2C8E68AE01479F545D55EB21AF0B" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1c770e52177ed3071dd2afe6eddb8d31">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1902bb6f-9742-43c7-83cd-78dfc04ff927" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9b5aab5975c58ac3b83150e37659e28a" ns2:_="">
     <xsd:import namespace="1902bb6f-9742-43c7-83cd-78dfc04ff927"/>
@@ -2910,15 +2905,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -2926,6 +2912,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{49273989-39D9-4CED-AEC6-610F5F9774BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81B62ADE-CE3E-4F60-A1C6-EF22221087A3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2939,14 +2933,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{49273989-39D9-4CED-AEC6-610F5F9774BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>